<commit_message>
fix: fallos de operacion que terminaban bien, tests de parada en la CI, rutas de los .ps1 y documentacion alineada con la evidencia (auditoria integral A10-A12, A16, A18, A21, A22, A25, A27, A28, A32, A38, A39, A44, A46, A47; Antigravity CI-01, CI-02, OPS-01, DOC-03)
</commit_message>
<xml_diff>
--- a/experimentos/plan_financiero/salida/detalle_v11.xlsx
+++ b/experimentos/plan_financiero/salida/detalle_v11.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance momento 0" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance año 1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance año 2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance año 3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados agregada" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados año 1" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados año 2" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados año 3" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tesorería año 1" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tesorería año 2" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tesorería año 3" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mensual" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balances" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Balance momento 0" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Balance año 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Balance año 2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Balance año 3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Resultados agregada" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Resultados año 1" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Resultados año 2" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Resultados año 3" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Tesorería año 1" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Tesorería año 2" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Tesorería año 3" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Mensual" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Balances" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Supuestos" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1395,13 +1395,13 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>7389.333125</v>
+        <v>7389.333124999999</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>7597.377500000001</v>
+        <v>7597.3775</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>7597.377500000001</v>
+        <v>7597.3775</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>7805.421875</v>
@@ -1410,22 +1410,22 @@
         <v>7805.421875</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>8013.46625</v>
+        <v>8013.466249999999</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>8013.46625</v>
+        <v>8013.466249999999</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>8221.510625000001</v>
+        <v>8221.510624999999</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>8013.46625</v>
+        <v>8013.466249999999</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>8221.510625000001</v>
+        <v>8221.510624999999</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>8221.510625000001</v>
+        <v>8221.510624999999</v>
       </c>
       <c r="M17" s="2" t="n">
         <v>8429.555</v>
@@ -1576,7 +1576,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>3264.699375000001</v>
+        <v>3264.699375000002</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
@@ -2012,7 +2012,7 @@
         <v>342982.244375</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>319324.6768749999</v>
+        <v>319324.676875</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>335277.2356944444</v>
@@ -3200,19 +3200,19 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>319232.0866666666</v>
+        <v>319232.0866666667</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>305620.4719444444</v>
+        <v>305620.4719444445</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>327154.5697916666</v>
+        <v>327154.5697916667</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>319465.3964583333</v>
+        <v>319465.3964583334</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>329220.9638194444</v>
+        <v>329220.9638194445</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>374122.24375</v>
@@ -7921,7 +7921,7 @@
         <v>3650</v>
       </c>
       <c r="X20" t="n">
-        <v>363954.82</v>
+        <v>363954.81</v>
       </c>
     </row>
     <row r="21">
@@ -8187,10 +8187,10 @@
         <v>-14248.62</v>
       </c>
       <c r="N24" t="n">
-        <v>225235.13</v>
+        <v>225235.12</v>
       </c>
       <c r="O24" t="n">
-        <v>260235.13</v>
+        <v>260235.12</v>
       </c>
       <c r="P24" t="n">
         <v>2000</v>
@@ -8557,10 +8557,10 @@
         <v>1759.58</v>
       </c>
       <c r="N29" t="n">
-        <v>230618.88</v>
+        <v>230618.87</v>
       </c>
       <c r="O29" t="n">
-        <v>265618.88</v>
+        <v>265618.87</v>
       </c>
       <c r="P29" t="n">
         <v>2000</v>
@@ -10193,7 +10193,7 @@
         </is>
       </c>
       <c r="K17" s="2" t="n">
-        <v>-46016.25</v>
+        <v>-46016.25000000003</v>
       </c>
     </row>
     <row r="18">
@@ -10580,7 +10580,7 @@
         </is>
       </c>
       <c r="K17" s="2" t="n">
-        <v>-56640.70833333334</v>
+        <v>-56640.7083333334</v>
       </c>
     </row>
     <row r="18">
@@ -11035,10 +11035,10 @@
         <v>31200</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>56800</v>
+        <v>56800.00000000001</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>75600</v>
+        <v>75600.00000000001</v>
       </c>
     </row>
     <row r="15">
@@ -11188,7 +11188,7 @@
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>Impuesto de sociedades (25 %, con las bases negativas compensadas)</t>
+          <t>Impuesto de sociedades (15 %, con las bases negativas compensadas)</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -12194,7 +12194,7 @@
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>Impuesto de sociedades (25 %, con las bases negativas compensadas)</t>
+          <t>Impuesto de sociedades (15 %, con las bases negativas compensadas)</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -13358,7 +13358,7 @@
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>Impuesto de sociedades (25 %, con las bases negativas compensadas)</t>
+          <t>Impuesto de sociedades (15 %, con las bases negativas compensadas)</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -14060,40 +14060,40 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>6300</v>
+        <v>6300.000000000001</v>
       </c>
       <c r="O14" s="3">
         <f>SUM(C14:N14)</f>
@@ -14522,7 +14522,7 @@
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>Impuesto de sociedades (25 %, con las bases negativas compensadas)</t>
+          <t>Impuesto de sociedades (15 %, con las bases negativas compensadas)</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">

</xml_diff>